<commit_message>
fix: pin seed dates to a fixed anchor so reseeding never moves them
prisma/seed.ts built every date as today + n days, so each reseed of the
shared database shifted all events, bookings and blocks, and the dates in
docs/test-cases/ went stale. day(n) is now 2026-09-26 + n days in Singapore
time, independent of the run date and the seeder's time zone.
SEED_ANCHOR=YYYY-MM-DD still overrides it for a one-off local run.

Re-based the seed-dependent dates in SPM-39 (+6 days), SPM-41 (+3) and
SPM-47 (+10), JSON and xlsx, which were written against 20, 23 and 16 Sep.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-39_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-39_Test_Cases.xlsx
@@ -498,6 +498,7 @@
       <c r="E1" s="8" t="n"/>
       <c r="F1" s="9" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1298,6 +1299,8 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
@@ -1476,6 +1479,7 @@
       </c>
       <c r="F37" s="9" t="n"/>
     </row>
+    <row r="38"/>
     <row r="39" ht="179.5" customHeight="1">
       <c r="A39" s="7" t="inlineStr">
         <is>
@@ -1507,8 +1511,8 @@
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B33:D33"/>
+    <mergeCell ref="E35:F35"/>
     <mergeCell ref="E34:F34"/>
-    <mergeCell ref="E35:F35"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="E30:F30"/>
     <mergeCell ref="B37:D37"/>
@@ -1664,6 +1668,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -1828,6 +1833,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -1994,6 +2000,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2157,6 +2164,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2319,6 +2327,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2483,6 +2492,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2647,6 +2657,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2813,6 +2824,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2979,6 +2991,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3075,7 +3088,7 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Demo data freshly loaded — no flag can be cleared from the app, so reload the demo data before this test.
-One-North Seminar Room (ONE-SEM) seats 80 theatre-style and has one approved future booking: 'Tanjong Legal CPD Seminar' on 28 Oct 2026, whose event expects 70 people. Its coordinator is Joel Fernandez.
+One-North Seminar Room (ONE-SEM) seats 80 theatre-style and has one approved future booking: 'Tanjong Legal CPD Seminar' on 3 Nov 2026, whose event expects 70 people. Its coordinator is Joel Fernandez.
 Logged in as Venue Staff: marcus.wong@connectsphere.com / password123</t>
         </is>
       </c>
@@ -3143,6 +3156,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3396,7 +3410,7 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Demo data freshly loaded.
-One-North Auditorium (ONE-AUD) seats 180 theatre-style and has one approved future booking: 'Bayu Energy Transition Panel' on 3 Nov 2026, whose event expects 160 people.
+One-North Auditorium (ONE-AUD) seats 180 theatre-style and has one approved future booking: 'Bayu Energy Transition Panel' on 9 Nov 2026, whose event expects 160 people.
 Logged in as Venue Staff: marcus.wong@connectsphere.com / password123</t>
         </is>
       </c>
@@ -3462,6 +3476,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3623,6 +3638,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3719,7 +3735,7 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Demo data freshly loaded.
-Changi Conference Centre (CBP-CONF) has one APPROVED future booking, 'Anchorpoint Supply Chain Briefing' on 20 Oct 2026, and one PENDING future booking, 'Pearl Delta Safety Conference'.
+Changi Conference Centre (CBP-CONF) has one APPROVED future booking, 'Anchorpoint Supply Chain Briefing' on 26 Oct 2026, and one PENDING future booking, 'Pearl Delta Safety Conference'.
 Logged in as Venue Staff: marcus.wong@connectsphere.com / password123</t>
         </is>
       </c>
@@ -3788,6 +3804,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3884,7 +3901,7 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Demo data freshly loaded.
-Jurong Training Room (JUR-TRN) has one approved FUTURE booking, 'Harbourline Claims Systems Training' on 13 Oct 2026, and one approved PAST booking, 'Meridian Compliance Training' from 25 Aug 2026.
+Jurong Training Room (JUR-TRN) has one approved FUTURE booking, 'Harbourline Claims Systems Training' on 19 Oct 2026, and one approved PAST booking, 'Meridian Compliance Training' from 31 Aug 2026.
 Logged in as Venue Staff: marcus.wong@connectsphere.com / password123</t>
         </is>
       </c>
@@ -3952,6 +3969,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -4119,6 +4137,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -4215,7 +4234,7 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Demo data freshly loaded.
-Jurong Expo Floor (JUR-EXP) has one approved future booking, 'Sundara Hospitality Trade Showcase' on 24 Nov 2026, whose event requires Loading bay access as a mandatory facility. Its coordinator is Daniel Tan.
+Jurong Expo Floor (JUR-EXP) has one approved future booking, 'Sundara Hospitality Trade Showcase' on 30 Nov 2026, whose event requires Loading bay access as a mandatory facility. Its coordinator is Daniel Tan.
 Logged in as Venue Staff: marcus.wong@connectsphere.com / password123</t>
         </is>
       </c>
@@ -4282,6 +4301,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -4444,6 +4464,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -4609,6 +4630,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -4774,6 +4796,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -4939,6 +4962,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -5101,6 +5125,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -5272,6 +5297,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -5438,6 +5464,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -5604,6 +5631,7 @@
         <v>46285</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>

</xml_diff>